<commit_message>
Kerki 33 + rank/value delta arrows
- Add Kerki 33 results (Quickracer10 W1, PandaMane, RoundNzt, microways, JakeAdjacent)
- New players: Renergy, add Yolo alias for Hi Im Yolo
- Rolling and Skill tabs now show rank movement arrows and points/mu deltas
- Build script reads previous kerki.json to embed prev_rank/prev_points/prev_mu
</commit_message>
<xml_diff>
--- a/Kerki Comp Results 31+.xlsx
+++ b/Kerki Comp Results 31+.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -427,6 +427,11 @@
           <t>27/3/26</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>12/4/26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -439,6 +444,11 @@
           <t>Kerki Comp #32- csc-ki</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Kerki Comp #33- Maps by Lexer, Victor, Tommygaming</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -471,6 +481,21 @@
           <t>Points</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Placement</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Points</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -479,6 +504,11 @@
         </is>
       </c>
       <c r="G4" t="inlineStr">
+        <is>
+          <t>Winners</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
         <is>
           <t>Winners</t>
         </is>
@@ -501,6 +531,14 @@
           <t>Kernkob</t>
         </is>
       </c>
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Quickracer10</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -519,6 +557,14 @@
           <t>PandaMane</t>
         </is>
       </c>
+      <c r="M6" t="n">
+        <v>2</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>PandaMane</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -537,6 +583,14 @@
           <t>RoundNzt</t>
         </is>
       </c>
+      <c r="M7" t="n">
+        <v>3</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>RoundNzt</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -555,6 +609,14 @@
           <t>MackCheesy</t>
         </is>
       </c>
+      <c r="M8" t="n">
+        <v>4</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>microways</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -573,6 +635,14 @@
           <t>Sandals</t>
         </is>
       </c>
+      <c r="M9" t="n">
+        <v>5</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>JakeAdjacent</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -581,6 +651,11 @@
         </is>
       </c>
       <c r="G10" t="inlineStr">
+        <is>
+          <t>Finalists</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
         <is>
           <t>Finalists</t>
         </is>
@@ -603,6 +678,14 @@
           <t>microways</t>
         </is>
       </c>
+      <c r="M11" t="n">
+        <v>1</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Job</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -621,6 +704,14 @@
           <t>quickracer</t>
         </is>
       </c>
+      <c r="M12" t="n">
+        <v>2</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>agix</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -631,6 +722,14 @@
           <t>St Nic</t>
         </is>
       </c>
+      <c r="M13" t="n">
+        <v>3</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Sterben</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -641,6 +740,14 @@
           <t>microways</t>
         </is>
       </c>
+      <c r="M14" t="n">
+        <v>4</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>brrryy</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -651,6 +758,14 @@
           <t>PandaMane</t>
         </is>
       </c>
+      <c r="M15" t="n">
+        <v>5</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Renergy</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -661,6 +776,14 @@
           <t>Lexer</t>
         </is>
       </c>
+      <c r="M16" t="n">
+        <v>6</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>M4rv</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -671,6 +794,14 @@
           <t>MackCheesy</t>
         </is>
       </c>
+      <c r="M17" t="n">
+        <v>7</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Hi Im Yolo</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -679,6 +810,14 @@
       <c r="B18" t="inlineStr">
         <is>
           <t>MALIYO</t>
+        </is>
+      </c>
+      <c r="M18" t="n">
+        <v>8</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Kernkob</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Kerki 33 full lobby + nuisance handling
- Add Others section for Kerki 33 (29 players, from Lexer screenshots)
- Add Nuisance section support to build script — mappers/playtesters marked
  as nuisance are excluded from stats per kerki (not counted toward apps,
  rankings, or skill ratings)
- Kerki 33 nuisances: justMaki (playtester), Victor + Tommygaming (mappers)
- Add ~20 new player canonicals cross-referenced against COTD + GTR data
</commit_message>
<xml_diff>
--- a/Kerki Comp Results 31+.xlsx
+++ b/Kerki Comp Results 31+.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O19"/>
+  <dimension ref="A1:O59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -830,7 +830,351 @@
           <t>Orthros</t>
         </is>
       </c>
-    </row>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="M20" t="n">
+        <v>1</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>MrBunny_666</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="M21" t="n">
+        <v>2</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>rtube</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="M22" t="n">
+        <v>3</v>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Noxitu</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="M23" t="n">
+        <v>4</v>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>aizpun</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="M24" t="n">
+        <v>5</v>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>wokonbike</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="M25" t="n">
+        <v>6</v>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>LoudSentinel</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="M26" t="n">
+        <v>7</v>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Six</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="M27" t="n">
+        <v>8</v>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Eclipse135</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="M28" t="n">
+        <v>9</v>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>PlusMicron</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="M29" t="n">
+        <v>10</v>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>redal</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="M30" t="n">
+        <v>11</v>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Shadynook</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="M31" t="n">
+        <v>12</v>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>376</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="M32" t="n">
+        <v>13</v>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>SharKy</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="M33" t="n">
+        <v>14</v>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>graysonvitek88</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="M34" t="n">
+        <v>15</v>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Heart-TGV</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="M35" t="n">
+        <v>16</v>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>DeeDeeNaNaNa</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="M36" t="n">
+        <v>17</v>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>LArk</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="M37" t="n">
+        <v>18</v>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Tudge Boat</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="M38" t="n">
+        <v>19</v>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Matic_D</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="M39" t="n">
+        <v>20</v>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>FedtStensDyr</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="M40" t="n">
+        <v>21</v>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>DorthJohson</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="M41" t="n">
+        <v>22</v>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>timesprout</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="M42" t="n">
+        <v>23</v>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>lil_zwimpie</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="M43" t="n">
+        <v>24</v>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Unfortunate Inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="M44" t="n">
+        <v>25</v>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>FlyBoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="M45" t="n">
+        <v>26</v>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>Smullie</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="M46" t="n">
+        <v>27</v>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>Sandals</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="M47" t="n">
+        <v>28</v>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>logix</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="M48" t="n">
+        <v>29</v>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>GuillaumePN</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>Nuisance</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>Sandals</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="M50" t="n">
+        <v>1</v>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>justMaki</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="M51" t="n">
+        <v>2</v>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>Victor</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="M52" t="n">
+        <v>3</v>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>Tommygaming</t>
+        </is>
+      </c>
+    </row>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Kerki #34 + Records tab deltas
</commit_message>
<xml_diff>
--- a/Kerki Comp Results 31+.xlsx
+++ b/Kerki Comp Results 31+.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O59"/>
+  <dimension ref="A1:U52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,6 +432,11 @@
           <t>12/4/26</t>
         </is>
       </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>26/4/26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -449,6 +454,11 @@
           <t>Kerki Comp #33- Maps by Lexer, Victor, Tommygaming</t>
         </is>
       </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Kerki Comp #34 - Maps by Maki, Shadynook, Redal</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -496,6 +506,21 @@
           <t>Points</t>
         </is>
       </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Placement</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Points</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -509,6 +534,11 @@
         </is>
       </c>
       <c r="M4" t="inlineStr">
+        <is>
+          <t>Winners</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
         <is>
           <t>Winners</t>
         </is>
@@ -539,6 +569,14 @@
           <t>Quickracer10</t>
         </is>
       </c>
+      <c r="S5" t="n">
+        <v>1</v>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>JakeAdjacent</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -565,6 +603,14 @@
           <t>PandaMane</t>
         </is>
       </c>
+      <c r="S6" t="n">
+        <v>2</v>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>PandaMane</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -591,6 +637,14 @@
           <t>RoundNzt</t>
         </is>
       </c>
+      <c r="S7" t="n">
+        <v>3</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>RoundNzt</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -617,6 +671,14 @@
           <t>microways</t>
         </is>
       </c>
+      <c r="S8" t="n">
+        <v>4</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Quickracer10</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -643,6 +705,14 @@
           <t>JakeAdjacent</t>
         </is>
       </c>
+      <c r="S9" t="n">
+        <v>5</v>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>ZOMAN</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -656,6 +726,11 @@
         </is>
       </c>
       <c r="M10" t="inlineStr">
+        <is>
+          <t>Finalists</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
         <is>
           <t>Finalists</t>
         </is>
@@ -686,6 +761,14 @@
           <t>Job</t>
         </is>
       </c>
+      <c r="S11" t="n">
+        <v>1</v>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Lexer</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -712,6 +795,14 @@
           <t>agix</t>
         </is>
       </c>
+      <c r="S12" t="n">
+        <v>2</v>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>Sandals</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -730,6 +821,14 @@
           <t>Sterben</t>
         </is>
       </c>
+      <c r="S13" t="n">
+        <v>3</v>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>rtube</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -748,6 +847,14 @@
           <t>brrryy</t>
         </is>
       </c>
+      <c r="S14" t="n">
+        <v>4</v>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>ping</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -766,6 +873,11 @@
           <t>Renergy</t>
         </is>
       </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -784,6 +896,14 @@
           <t>M4rv</t>
         </is>
       </c>
+      <c r="S16" t="n">
+        <v>1</v>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Warsnac</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -802,6 +922,14 @@
           <t>Hi Im Yolo</t>
         </is>
       </c>
+      <c r="S17" t="n">
+        <v>2</v>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>JobW</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -820,6 +948,14 @@
           <t>Kernkob</t>
         </is>
       </c>
+      <c r="S18" t="n">
+        <v>3</v>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>icRS</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -835,6 +971,14 @@
           <t>Other</t>
         </is>
       </c>
+      <c r="S19" t="n">
+        <v>4</v>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>Victor</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="M20" t="n">
@@ -845,6 +989,14 @@
           <t>MrBunny_666</t>
         </is>
       </c>
+      <c r="S20" t="n">
+        <v>5</v>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>Diabler</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="M21" t="n">
@@ -855,6 +1007,14 @@
           <t>rtube</t>
         </is>
       </c>
+      <c r="S21" t="n">
+        <v>6</v>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>BB_Benji</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="M22" t="n">
@@ -865,6 +1025,14 @@
           <t>Noxitu</t>
         </is>
       </c>
+      <c r="S22" t="n">
+        <v>7</v>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>agix</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="M23" t="n">
@@ -875,6 +1043,14 @@
           <t>aizpun</t>
         </is>
       </c>
+      <c r="S23" t="n">
+        <v>8</v>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>Six</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="M24" t="n">
@@ -885,6 +1061,14 @@
           <t>wokonbike</t>
         </is>
       </c>
+      <c r="S24" t="n">
+        <v>9</v>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Heart-TGV</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="M25" t="n">
@@ -895,6 +1079,14 @@
           <t>LoudSentinel</t>
         </is>
       </c>
+      <c r="S25" t="n">
+        <v>10</v>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>Murrl</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="M26" t="n">
@@ -905,6 +1097,14 @@
           <t>Six</t>
         </is>
       </c>
+      <c r="S26" t="n">
+        <v>11</v>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>Stick</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="M27" t="n">
@@ -915,6 +1115,14 @@
           <t>Eclipse135</t>
         </is>
       </c>
+      <c r="S27" t="n">
+        <v>12</v>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>PlusMicron</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="M28" t="n">
@@ -925,6 +1133,14 @@
           <t>PlusMicron</t>
         </is>
       </c>
+      <c r="S28" t="n">
+        <v>13</v>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>Matic_D</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="M29" t="n">
@@ -935,6 +1151,14 @@
           <t>redal</t>
         </is>
       </c>
+      <c r="S29" t="n">
+        <v>14</v>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>MackCheesy</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="M30" t="n">
@@ -945,6 +1169,14 @@
           <t>Shadynook</t>
         </is>
       </c>
+      <c r="S30" t="n">
+        <v>15</v>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>FINSTER83</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="M31" t="n">
@@ -955,6 +1187,14 @@
           <t>376</t>
         </is>
       </c>
+      <c r="S31" t="n">
+        <v>16</v>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>K410K3N</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="M32" t="n">
@@ -965,6 +1205,14 @@
           <t>SharKy</t>
         </is>
       </c>
+      <c r="S32" t="n">
+        <v>17</v>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Noxitu</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="M33" t="n">
@@ -975,6 +1223,14 @@
           <t>graysonvitek88</t>
         </is>
       </c>
+      <c r="S33" t="n">
+        <v>18</v>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>R0nanC</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="M34" t="n">
@@ -985,6 +1241,14 @@
           <t>Heart-TGV</t>
         </is>
       </c>
+      <c r="S34" t="n">
+        <v>19</v>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>GuillaumePN</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="M35" t="n">
@@ -995,6 +1259,14 @@
           <t>DeeDeeNaNaNa</t>
         </is>
       </c>
+      <c r="S35" t="n">
+        <v>20</v>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>Form</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="M36" t="n">
@@ -1005,6 +1277,14 @@
           <t>LArk</t>
         </is>
       </c>
+      <c r="S36" t="n">
+        <v>21</v>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>imagineaclevernamehere</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="M37" t="n">
@@ -1015,6 +1295,14 @@
           <t>Tudge Boat</t>
         </is>
       </c>
+      <c r="S37" t="n">
+        <v>22</v>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>aizpun</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="M38" t="n">
@@ -1025,6 +1313,14 @@
           <t>Matic_D</t>
         </is>
       </c>
+      <c r="S38" t="n">
+        <v>23</v>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>lucanakin</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="M39" t="n">
@@ -1035,6 +1331,14 @@
           <t>FedtStensDyr</t>
         </is>
       </c>
+      <c r="S39" t="n">
+        <v>24</v>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>Fly8oy</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="M40" t="n">
@@ -1045,6 +1349,14 @@
           <t>DorthJohson</t>
         </is>
       </c>
+      <c r="S40" t="n">
+        <v>25</v>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>376</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="M41" t="n">
@@ -1055,6 +1367,14 @@
           <t>timesprout</t>
         </is>
       </c>
+      <c r="S41" t="n">
+        <v>26</v>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>timesprout</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="M42" t="n">
@@ -1065,6 +1385,14 @@
           <t>lil_zwimpie</t>
         </is>
       </c>
+      <c r="S42" t="n">
+        <v>27</v>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>M4DSCOTSM4N</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="M43" t="n">
@@ -1075,6 +1403,14 @@
           <t>Unfortunate Inc</t>
         </is>
       </c>
+      <c r="S43" t="n">
+        <v>28</v>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>Lynhardt</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="M44" t="n">
@@ -1085,6 +1421,14 @@
           <t>FlyBoy</t>
         </is>
       </c>
+      <c r="S44" t="n">
+        <v>29</v>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>wokonbike</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="M45" t="n">
@@ -1095,6 +1439,14 @@
           <t>Smullie</t>
         </is>
       </c>
+      <c r="S45" t="n">
+        <v>30</v>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>SKULL00</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="M46" t="n">
@@ -1105,6 +1457,14 @@
           <t>Sandals</t>
         </is>
       </c>
+      <c r="S46" t="n">
+        <v>31</v>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>Games_BS</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="M47" t="n">
@@ -1115,6 +1475,14 @@
           <t>logix</t>
         </is>
       </c>
+      <c r="S47" t="n">
+        <v>32</v>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>tacklesskoala8</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="M48" t="n">
@@ -1125,6 +1493,14 @@
           <t>GuillaumePN</t>
         </is>
       </c>
+      <c r="S48" t="n">
+        <v>33</v>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>Zeus</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="M49" t="inlineStr">
@@ -1135,6 +1511,14 @@
       <c r="N49" t="inlineStr">
         <is>
           <t>Sandals</t>
+        </is>
+      </c>
+      <c r="S49" t="n">
+        <v>34</v>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>sailingman</t>
         </is>
       </c>
     </row>
@@ -1168,13 +1552,6 @@
         </is>
       </c>
     </row>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mark PlusMicron as nuisance in Kerki #36 (mapped Strawberry Lemonade)
</commit_message>
<xml_diff>
--- a/Kerki Comp Results 31+.xlsx
+++ b/Kerki Comp Results 31+.xlsx
@@ -1967,7 +1967,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>24/5/26</t>
+          <t>26/5/26</t>
         </is>
       </c>
     </row>
@@ -2344,11 +2344,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PlusMicron</t>
+          <t>lil_zwimpie</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>310</v>
+        <v>285</v>
       </c>
     </row>
     <row r="36">
@@ -2357,11 +2357,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>lil_zwimpie</t>
+          <t>Noxitu</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>285</v>
+        <v>260</v>
       </c>
     </row>
     <row r="37">
@@ -2370,11 +2370,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Noxitu</t>
+          <t>LILWOOLEY</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>260</v>
+        <v>240</v>
       </c>
     </row>
     <row r="38">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>LILWOOLEY</t>
+          <t>BrickEdwards</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>240</v>
+        <v>225</v>
       </c>
     </row>
     <row r="39">
@@ -2396,11 +2396,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>BrickEdwards</t>
+          <t>M4DSCOTSM4N</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>225</v>
+        <v>190</v>
       </c>
     </row>
     <row r="40">
@@ -2409,11 +2409,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>M4DSCOTSM4N</t>
+          <t>Ritchi</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>190</v>
+        <v>185</v>
       </c>
     </row>
     <row r="41">
@@ -2422,11 +2422,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Ritchi</t>
+          <t>timesprout</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>185</v>
+        <v>165</v>
       </c>
     </row>
     <row r="42">
@@ -2435,11 +2435,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>timesprout</t>
+          <t>Wheelie</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="43">
@@ -2448,11 +2448,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Wheelie</t>
+          <t>MAGS3</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>160</v>
+        <v>65</v>
       </c>
     </row>
     <row r="44">
@@ -2461,11 +2461,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>MAGS3</t>
+          <t>cookie</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
     </row>
     <row r="45">
@@ -2474,44 +2474,44 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>cookie</t>
+          <t>groovy</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="n">
-        <v>26</v>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>groovy</t>
-        </is>
-      </c>
-      <c r="C46" t="n">
-        <v>30</v>
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Nuisance</t>
+        </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Nuisance</t>
-        </is>
+      <c r="A47" t="n">
+        <v>1</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Renergy</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>600</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Renergy</t>
+          <t>PlusMicron</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>600</v>
+        <v>310</v>
       </c>
     </row>
     <row r="49"/>

</xml_diff>

<commit_message>
Add Kerki #37 standings (maps by bjenk, Shattersmith, Maki)
Winners: microways, JakeAdjacent, rtube, Lexer, RoundNzt.
Finalists: Quickracer10, Sandals, Minkus, Hi Im Yolo, PlusMicron.

Discovery rounds were played before the logger was started, so the
log contains no warmup rounds. Added --no-warmup to parse_kerki_from_log.py
to score every round in that case; default warmup detection would have
discarded the first appearance of each map as discovery, docking ~3 rounds
of points from everyone and breaking winner/finalist detection. Parsed
results now match Maki's announced honors and the in-game cup-tracker totals.
</commit_message>
<xml_diff>
--- a/Kerki Comp Results 31+.xlsx
+++ b/Kerki Comp Results 31+.xlsx
@@ -1961,7 +1961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1970,6 +1970,11 @@
           <t>26/5/26</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>7/6/26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1977,6 +1982,11 @@
           <t>Kerki Comp #36 - Maps by Renergy, Ferret, PlusMicron</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Kerki Comp #37 - Maps by bjenk, Shattersmith, Maki</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1994,9 +2004,29 @@
           <t>Points</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Placement</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Points</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
+        <is>
+          <t>Winners</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>Winners</t>
         </is>
@@ -2011,6 +2041,14 @@
           <t>justMaki</t>
         </is>
       </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>microways</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -2021,6 +2059,14 @@
           <t>Kernkob</t>
         </is>
       </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>JakeAdjacent</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -2031,6 +2077,14 @@
           <t>Quickracer10</t>
         </is>
       </c>
+      <c r="G7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>rtube</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -2041,6 +2095,14 @@
           <t>Sterben</t>
         </is>
       </c>
+      <c r="G8" t="n">
+        <v>4</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Lexer</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -2051,9 +2113,22 @@
           <t>RoundNzt</t>
         </is>
       </c>
+      <c r="G9" t="n">
+        <v>5</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>RoundNzt</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
+        <is>
+          <t>Finalists</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
         <is>
           <t>Finalists</t>
         </is>
@@ -2068,6 +2143,14 @@
           <t>JakeAdjacent</t>
         </is>
       </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Quickracer10</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -2078,6 +2161,14 @@
           <t>Lexer</t>
         </is>
       </c>
+      <c r="G12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Sandals</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -2088,6 +2179,14 @@
           <t>Minkus</t>
         </is>
       </c>
+      <c r="G13" t="n">
+        <v>3</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Minkus</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -2098,6 +2197,14 @@
           <t>Stick</t>
         </is>
       </c>
+      <c r="G14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Hi Im Yolo</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -2108,6 +2215,14 @@
           <t>PandaMane</t>
         </is>
       </c>
+      <c r="G15" t="n">
+        <v>5</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>PlusMicron</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -2118,6 +2233,11 @@
           <t>ZOMAN</t>
         </is>
       </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2128,6 +2248,17 @@
           <t>ping</t>
         </is>
       </c>
+      <c r="G17" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>agix</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>750</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -2138,6 +2269,17 @@
           <t>microways</t>
         </is>
       </c>
+      <c r="G18" t="n">
+        <v>2</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>brrryy</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>750</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -2148,12 +2290,34 @@
           <t>brrryy</t>
         </is>
       </c>
+      <c r="G19" t="n">
+        <v>3</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Heart-TGV</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>750</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
+      </c>
+      <c r="G20" t="n">
+        <v>4</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>DeiRex</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>675</v>
       </c>
     </row>
     <row r="21">
@@ -2168,6 +2332,17 @@
       <c r="C21" t="n">
         <v>705</v>
       </c>
+      <c r="G21" t="n">
+        <v>5</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Wheelie</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>660</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -2181,6 +2356,17 @@
       <c r="C22" t="n">
         <v>700</v>
       </c>
+      <c r="G22" t="n">
+        <v>6</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Noxitu</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>630</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -2194,6 +2380,17 @@
       <c r="C23" t="n">
         <v>685</v>
       </c>
+      <c r="G23" t="n">
+        <v>7</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Matic_D</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>625</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -2207,6 +2404,17 @@
       <c r="C24" t="n">
         <v>680</v>
       </c>
+      <c r="G24" t="n">
+        <v>8</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>aizpun</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>620</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2220,6 +2428,17 @@
       <c r="C25" t="n">
         <v>680</v>
       </c>
+      <c r="G25" t="n">
+        <v>9</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>ZOMAN</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>570</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2233,6 +2452,17 @@
       <c r="C26" t="n">
         <v>675</v>
       </c>
+      <c r="G26" t="n">
+        <v>10</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Hellmet</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>475</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2246,6 +2476,17 @@
       <c r="C27" t="n">
         <v>665</v>
       </c>
+      <c r="G27" t="n">
+        <v>11</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>timesprout</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>400</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2259,6 +2500,17 @@
       <c r="C28" t="n">
         <v>650</v>
       </c>
+      <c r="G28" t="n">
+        <v>12</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Joe Beidl</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>355</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2272,6 +2524,17 @@
       <c r="C29" t="n">
         <v>595</v>
       </c>
+      <c r="G29" t="n">
+        <v>13</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>ping</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>355</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2285,6 +2548,17 @@
       <c r="C30" t="n">
         <v>565</v>
       </c>
+      <c r="G30" t="n">
+        <v>14</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Andrew8Kavanagh</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>345</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2298,6 +2572,17 @@
       <c r="C31" t="n">
         <v>505</v>
       </c>
+      <c r="G31" t="n">
+        <v>15</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>User Data</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>310</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2311,6 +2596,17 @@
       <c r="C32" t="n">
         <v>460</v>
       </c>
+      <c r="G32" t="n">
+        <v>16</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>MALIYO</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>280</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2324,6 +2620,17 @@
       <c r="C33" t="n">
         <v>425</v>
       </c>
+      <c r="G33" t="n">
+        <v>17</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>icRS</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>275</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2337,6 +2644,17 @@
       <c r="C34" t="n">
         <v>380</v>
       </c>
+      <c r="G34" t="n">
+        <v>18</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Waaksaam</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>255</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2350,6 +2668,17 @@
       <c r="C35" t="n">
         <v>285</v>
       </c>
+      <c r="G35" t="n">
+        <v>19</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>MetalCJ</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>215</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2363,6 +2692,17 @@
       <c r="C36" t="n">
         <v>260</v>
       </c>
+      <c r="G36" t="n">
+        <v>20</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>FINSTER83</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>180</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2376,6 +2716,17 @@
       <c r="C37" t="n">
         <v>240</v>
       </c>
+      <c r="G37" t="n">
+        <v>21</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>dtmittens</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>130</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2389,6 +2740,17 @@
       <c r="C38" t="n">
         <v>225</v>
       </c>
+      <c r="G38" t="n">
+        <v>22</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Darkblade</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>125</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2402,6 +2764,17 @@
       <c r="C39" t="n">
         <v>190</v>
       </c>
+      <c r="G39" t="n">
+        <v>23</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>liz1rd</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2415,6 +2788,17 @@
       <c r="C40" t="n">
         <v>185</v>
       </c>
+      <c r="G40" t="n">
+        <v>24</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>gianzubler</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2428,6 +2812,17 @@
       <c r="C41" t="n">
         <v>165</v>
       </c>
+      <c r="G41" t="n">
+        <v>25</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Nascarkid18</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2441,6 +2836,17 @@
       <c r="C42" t="n">
         <v>160</v>
       </c>
+      <c r="G42" t="n">
+        <v>26</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Proxy</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2454,6 +2860,11 @@
       <c r="C43" t="n">
         <v>65</v>
       </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Nuisance</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2467,6 +2878,17 @@
       <c r="C44" t="n">
         <v>60</v>
       </c>
+      <c r="G44" t="n">
+        <v>1</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>justMaki</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>1230</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2480,12 +2902,34 @@
       <c r="C45" t="n">
         <v>30</v>
       </c>
+      <c r="G45" t="n">
+        <v>2</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Shattersmith</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>755</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
           <t>Nuisance</t>
         </is>
+      </c>
+      <c r="G46" t="n">
+        <v>3</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>bjenk4</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>185</v>
       </c>
     </row>
     <row r="47">

</xml_diff>

<commit_message>
Add Kerki #38: Kernkob W1, JakeAdjacent W2, RoundNzt/Sterben/Quickracer10
</commit_message>
<xml_diff>
--- a/Kerki Comp Results 31+.xlsx
+++ b/Kerki Comp Results 31+.xlsx
@@ -1961,7 +1961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:O59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1975,6 +1975,11 @@
           <t>7/6/26</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>21/6/26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1987,6 +1992,11 @@
           <t>Kerki Comp #37 - Maps by bjenk, Shattersmith, Maki</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Kerki Comp #38 - Maps by Tommy, Shadynook, Noxitu</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2019,6 +2029,21 @@
           <t>Points</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Placement</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Points</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2027,6 +2052,11 @@
         </is>
       </c>
       <c r="G4" t="inlineStr">
+        <is>
+          <t>Winners</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
         <is>
           <t>Winners</t>
         </is>
@@ -2049,6 +2079,14 @@
           <t>microways</t>
         </is>
       </c>
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Kernkob</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -2067,6 +2105,14 @@
           <t>JakeAdjacent</t>
         </is>
       </c>
+      <c r="M6" t="n">
+        <v>2</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>JakeAdjacent</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -2085,6 +2131,14 @@
           <t>rtube</t>
         </is>
       </c>
+      <c r="M7" t="n">
+        <v>3</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>RoundNzt</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -2103,6 +2157,14 @@
           <t>Lexer</t>
         </is>
       </c>
+      <c r="M8" t="n">
+        <v>4</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Sterben</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -2121,6 +2183,14 @@
           <t>RoundNzt</t>
         </is>
       </c>
+      <c r="M9" t="n">
+        <v>5</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Quickracer10</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2129,6 +2199,11 @@
         </is>
       </c>
       <c r="G10" t="inlineStr">
+        <is>
+          <t>Finalists</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
         <is>
           <t>Finalists</t>
         </is>
@@ -2151,6 +2226,14 @@
           <t>Quickracer10</t>
         </is>
       </c>
+      <c r="M11" t="n">
+        <v>1</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>microways</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -2169,6 +2252,14 @@
           <t>Sandals</t>
         </is>
       </c>
+      <c r="M12" t="n">
+        <v>2</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Lexer</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -2187,6 +2278,14 @@
           <t>Minkus</t>
         </is>
       </c>
+      <c r="M13" t="n">
+        <v>3</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Minkus</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -2205,6 +2304,11 @@
           <t>Hi Im Yolo</t>
         </is>
       </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -2223,6 +2327,17 @@
           <t>PlusMicron</t>
         </is>
       </c>
+      <c r="M15" t="n">
+        <v>1</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>PlusMicron</t>
+        </is>
+      </c>
+      <c r="O15" t="n">
+        <v>750</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -2238,6 +2353,17 @@
           <t>Other</t>
         </is>
       </c>
+      <c r="M16" t="n">
+        <v>2</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Six</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
+        <v>720</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2259,6 +2385,17 @@
       <c r="I17" t="n">
         <v>750</v>
       </c>
+      <c r="M17" t="n">
+        <v>3</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>MALIYO</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>705</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -2280,6 +2417,17 @@
       <c r="I18" t="n">
         <v>750</v>
       </c>
+      <c r="M18" t="n">
+        <v>4</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Diabler</t>
+        </is>
+      </c>
+      <c r="O18" t="n">
+        <v>675</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -2301,6 +2449,17 @@
       <c r="I19" t="n">
         <v>750</v>
       </c>
+      <c r="M19" t="n">
+        <v>5</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Matic_D</t>
+        </is>
+      </c>
+      <c r="O19" t="n">
+        <v>675</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2318,6 +2477,17 @@
       </c>
       <c r="I20" t="n">
         <v>675</v>
+      </c>
+      <c r="M20" t="n">
+        <v>6</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>agix</t>
+        </is>
+      </c>
+      <c r="O20" t="n">
+        <v>665</v>
       </c>
     </row>
     <row r="21">
@@ -2343,6 +2513,17 @@
       <c r="I21" t="n">
         <v>660</v>
       </c>
+      <c r="M21" t="n">
+        <v>7</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>FINSTER83</t>
+        </is>
+      </c>
+      <c r="O21" t="n">
+        <v>655</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -2367,6 +2548,17 @@
       <c r="I22" t="n">
         <v>630</v>
       </c>
+      <c r="M22" t="n">
+        <v>8</v>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Joe Beidl</t>
+        </is>
+      </c>
+      <c r="O22" t="n">
+        <v>605</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -2391,6 +2583,17 @@
       <c r="I23" t="n">
         <v>625</v>
       </c>
+      <c r="M23" t="n">
+        <v>9</v>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>aizpun</t>
+        </is>
+      </c>
+      <c r="O23" t="n">
+        <v>510</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -2415,6 +2618,17 @@
       <c r="I24" t="n">
         <v>620</v>
       </c>
+      <c r="M24" t="n">
+        <v>10</v>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>SjorsTea</t>
+        </is>
+      </c>
+      <c r="O24" t="n">
+        <v>480</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2439,6 +2653,17 @@
       <c r="I25" t="n">
         <v>570</v>
       </c>
+      <c r="M25" t="n">
+        <v>11</v>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>TheRockingSheep</t>
+        </is>
+      </c>
+      <c r="O25" t="n">
+        <v>480</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2463,6 +2688,17 @@
       <c r="I26" t="n">
         <v>475</v>
       </c>
+      <c r="M26" t="n">
+        <v>12</v>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Heart-TGV</t>
+        </is>
+      </c>
+      <c r="O26" t="n">
+        <v>455</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2487,6 +2723,17 @@
       <c r="I27" t="n">
         <v>400</v>
       </c>
+      <c r="M27" t="n">
+        <v>13</v>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Samueras</t>
+        </is>
+      </c>
+      <c r="O27" t="n">
+        <v>450</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2511,6 +2758,17 @@
       <c r="I28" t="n">
         <v>355</v>
       </c>
+      <c r="M28" t="n">
+        <v>14</v>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>wunderBarr</t>
+        </is>
+      </c>
+      <c r="O28" t="n">
+        <v>445</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2535,6 +2793,17 @@
       <c r="I29" t="n">
         <v>355</v>
       </c>
+      <c r="M29" t="n">
+        <v>15</v>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>wokonbike</t>
+        </is>
+      </c>
+      <c r="O29" t="n">
+        <v>415</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2559,6 +2828,17 @@
       <c r="I30" t="n">
         <v>345</v>
       </c>
+      <c r="M30" t="n">
+        <v>16</v>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Murrl</t>
+        </is>
+      </c>
+      <c r="O30" t="n">
+        <v>410</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2583,6 +2863,17 @@
       <c r="I31" t="n">
         <v>310</v>
       </c>
+      <c r="M31" t="n">
+        <v>17</v>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>M4DSCOTSM4N</t>
+        </is>
+      </c>
+      <c r="O31" t="n">
+        <v>380</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2607,6 +2898,17 @@
       <c r="I32" t="n">
         <v>280</v>
       </c>
+      <c r="M32" t="n">
+        <v>18</v>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Hellmet</t>
+        </is>
+      </c>
+      <c r="O32" t="n">
+        <v>370</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2631,6 +2933,17 @@
       <c r="I33" t="n">
         <v>275</v>
       </c>
+      <c r="M33" t="n">
+        <v>19</v>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>SuperHeavy</t>
+        </is>
+      </c>
+      <c r="O33" t="n">
+        <v>325</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2655,6 +2968,17 @@
       <c r="I34" t="n">
         <v>255</v>
       </c>
+      <c r="M34" t="n">
+        <v>20</v>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>timesprout</t>
+        </is>
+      </c>
+      <c r="O34" t="n">
+        <v>315</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2679,6 +3003,17 @@
       <c r="I35" t="n">
         <v>215</v>
       </c>
+      <c r="M35" t="n">
+        <v>21</v>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>''</t>
+        </is>
+      </c>
+      <c r="O35" t="n">
+        <v>300</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2703,6 +3038,17 @@
       <c r="I36" t="n">
         <v>180</v>
       </c>
+      <c r="M36" t="n">
+        <v>22</v>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Fly8oy</t>
+        </is>
+      </c>
+      <c r="O36" t="n">
+        <v>285</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2727,6 +3073,17 @@
       <c r="I37" t="n">
         <v>130</v>
       </c>
+      <c r="M37" t="n">
+        <v>23</v>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>martinsvalley</t>
+        </is>
+      </c>
+      <c r="O37" t="n">
+        <v>215</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2751,6 +3108,17 @@
       <c r="I38" t="n">
         <v>125</v>
       </c>
+      <c r="M38" t="n">
+        <v>24</v>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Orb Bee Bob</t>
+        </is>
+      </c>
+      <c r="O38" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2775,6 +3143,17 @@
       <c r="I39" t="n">
         <v>100</v>
       </c>
+      <c r="M39" t="n">
+        <v>25</v>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>tcrroadie</t>
+        </is>
+      </c>
+      <c r="O39" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2799,6 +3178,17 @@
       <c r="I40" t="n">
         <v>90</v>
       </c>
+      <c r="M40" t="n">
+        <v>26</v>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Darkblade</t>
+        </is>
+      </c>
+      <c r="O40" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2823,6 +3213,17 @@
       <c r="I41" t="n">
         <v>30</v>
       </c>
+      <c r="M41" t="n">
+        <v>27</v>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Don_E [GER]</t>
+        </is>
+      </c>
+      <c r="O41" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2847,6 +3248,11 @@
       <c r="I42" t="n">
         <v>30</v>
       </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>Nuisance</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2865,6 +3271,17 @@
           <t>Nuisance</t>
         </is>
       </c>
+      <c r="M43" t="n">
+        <v>1</v>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>justMaki</t>
+        </is>
+      </c>
+      <c r="O43" t="n">
+        <v>860</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2889,6 +3306,17 @@
       <c r="I44" t="n">
         <v>1230</v>
       </c>
+      <c r="M44" t="n">
+        <v>2</v>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Noxitu</t>
+        </is>
+      </c>
+      <c r="O44" t="n">
+        <v>485</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2913,6 +3341,17 @@
       <c r="I45" t="n">
         <v>755</v>
       </c>
+      <c r="M45" t="n">
+        <v>3</v>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>Tommygaming</t>
+        </is>
+      </c>
+      <c r="O45" t="n">
+        <v>370</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2930,6 +3369,17 @@
       </c>
       <c r="I46" t="n">
         <v>185</v>
+      </c>
+      <c r="M46" t="n">
+        <v>4</v>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>Shadynook</t>
+        </is>
+      </c>
+      <c r="O46" t="n">
+        <v>355</v>
       </c>
     </row>
     <row r="47">

</xml_diff>

<commit_message>
Add Kerki #39: Kernkob W1 clinches the K31+ season; parser gains --maps/--discovered ask-first warmup handling
</commit_message>
<xml_diff>
--- a/Kerki Comp Results 31+.xlsx
+++ b/Kerki Comp Results 31+.xlsx
@@ -1961,7 +1961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O59"/>
+  <dimension ref="A1:U59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1980,6 +1980,11 @@
           <t>21/6/26</t>
         </is>
       </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>5/7/26</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1997,6 +2002,11 @@
           <t>Kerki Comp #38 - Maps by Tommy, Shadynook, Noxitu</t>
         </is>
       </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Kerki Comp #39 - Maps by brrryy, Draugur, Shattersmith &amp; IronDragon</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2044,6 +2054,21 @@
           <t>Points</t>
         </is>
       </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Placement</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Points</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2057,6 +2082,11 @@
         </is>
       </c>
       <c r="M4" t="inlineStr">
+        <is>
+          <t>Winners</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
         <is>
           <t>Winners</t>
         </is>
@@ -2087,6 +2117,14 @@
           <t>Kernkob</t>
         </is>
       </c>
+      <c r="S5" t="n">
+        <v>1</v>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Kernkob</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -2113,6 +2151,14 @@
           <t>JakeAdjacent</t>
         </is>
       </c>
+      <c r="S6" t="n">
+        <v>2</v>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Jake</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -2139,6 +2185,14 @@
           <t>RoundNzt</t>
         </is>
       </c>
+      <c r="S7" t="n">
+        <v>3</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Lexer</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -2165,6 +2219,14 @@
           <t>Sterben</t>
         </is>
       </c>
+      <c r="S8" t="n">
+        <v>4</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Quickracer10</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -2191,6 +2253,14 @@
           <t>Quickracer10</t>
         </is>
       </c>
+      <c r="S9" t="n">
+        <v>5</v>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>PandaMane</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2204,6 +2274,11 @@
         </is>
       </c>
       <c r="M10" t="inlineStr">
+        <is>
+          <t>Finalists</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
         <is>
           <t>Finalists</t>
         </is>
@@ -2234,6 +2309,14 @@
           <t>microways</t>
         </is>
       </c>
+      <c r="S11" t="n">
+        <v>1</v>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Sterben</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -2260,6 +2343,14 @@
           <t>Lexer</t>
         </is>
       </c>
+      <c r="S12" t="n">
+        <v>2</v>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>RoundNzt</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -2286,6 +2377,14 @@
           <t>Minkus</t>
         </is>
       </c>
+      <c r="S13" t="n">
+        <v>3</v>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>Minkus</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -2309,6 +2408,14 @@
           <t>Other</t>
         </is>
       </c>
+      <c r="S14" t="n">
+        <v>4</v>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>Linzi</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -2338,6 +2445,14 @@
       <c r="O15" t="n">
         <v>750</v>
       </c>
+      <c r="S15" t="n">
+        <v>5</v>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>MALIYO</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -2364,6 +2479,14 @@
       <c r="O16" t="n">
         <v>720</v>
       </c>
+      <c r="S16" t="n">
+        <v>6</v>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>microways</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2396,6 +2519,11 @@
       <c r="O17" t="n">
         <v>705</v>
       </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -2428,6 +2556,17 @@
       <c r="O18" t="n">
         <v>675</v>
       </c>
+      <c r="S18" t="n">
+        <v>1</v>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>agix</t>
+        </is>
+      </c>
+      <c r="U18" t="n">
+        <v>750</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -2460,6 +2599,17 @@
       <c r="O19" t="n">
         <v>675</v>
       </c>
+      <c r="S19" t="n">
+        <v>2</v>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>Heart-TGV</t>
+        </is>
+      </c>
+      <c r="U19" t="n">
+        <v>750</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2488,6 +2638,17 @@
       </c>
       <c r="O20" t="n">
         <v>665</v>
+      </c>
+      <c r="S20" t="n">
+        <v>3</v>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>ferinine</t>
+        </is>
+      </c>
+      <c r="U20" t="n">
+        <v>730</v>
       </c>
     </row>
     <row r="21">
@@ -2524,6 +2685,17 @@
       <c r="O21" t="n">
         <v>655</v>
       </c>
+      <c r="S21" t="n">
+        <v>4</v>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>Savage Package</t>
+        </is>
+      </c>
+      <c r="U21" t="n">
+        <v>720</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -2559,6 +2731,17 @@
       <c r="O22" t="n">
         <v>605</v>
       </c>
+      <c r="S22" t="n">
+        <v>5</v>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Tommygaming</t>
+        </is>
+      </c>
+      <c r="U22" t="n">
+        <v>720</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -2594,6 +2777,17 @@
       <c r="O23" t="n">
         <v>510</v>
       </c>
+      <c r="S23" t="n">
+        <v>6</v>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>Noxitu</t>
+        </is>
+      </c>
+      <c r="U23" t="n">
+        <v>670</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -2629,6 +2823,17 @@
       <c r="O24" t="n">
         <v>480</v>
       </c>
+      <c r="S24" t="n">
+        <v>7</v>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Kiprosa</t>
+        </is>
+      </c>
+      <c r="U24" t="n">
+        <v>595</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2664,6 +2869,17 @@
       <c r="O25" t="n">
         <v>480</v>
       </c>
+      <c r="S25" t="n">
+        <v>8</v>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>Joe Beidl</t>
+        </is>
+      </c>
+      <c r="U25" t="n">
+        <v>580</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2699,6 +2915,17 @@
       <c r="O26" t="n">
         <v>455</v>
       </c>
+      <c r="S26" t="n">
+        <v>9</v>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>wokonbike</t>
+        </is>
+      </c>
+      <c r="U26" t="n">
+        <v>580</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2734,6 +2961,17 @@
       <c r="O27" t="n">
         <v>450</v>
       </c>
+      <c r="S27" t="n">
+        <v>10</v>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>daytime</t>
+        </is>
+      </c>
+      <c r="U27" t="n">
+        <v>565</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2769,6 +3007,17 @@
       <c r="O28" t="n">
         <v>445</v>
       </c>
+      <c r="S28" t="n">
+        <v>11</v>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>elekvault</t>
+        </is>
+      </c>
+      <c r="U28" t="n">
+        <v>560</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2804,6 +3053,17 @@
       <c r="O29" t="n">
         <v>415</v>
       </c>
+      <c r="S29" t="n">
+        <v>12</v>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>TheRockingSheep</t>
+        </is>
+      </c>
+      <c r="U29" t="n">
+        <v>550</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2839,6 +3099,17 @@
       <c r="O30" t="n">
         <v>410</v>
       </c>
+      <c r="S30" t="n">
+        <v>13</v>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>St Nicholas</t>
+        </is>
+      </c>
+      <c r="U30" t="n">
+        <v>540</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2874,6 +3145,17 @@
       <c r="O31" t="n">
         <v>380</v>
       </c>
+      <c r="S31" t="n">
+        <v>14</v>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>SuperHeavy</t>
+        </is>
+      </c>
+      <c r="U31" t="n">
+        <v>535</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2909,6 +3191,17 @@
       <c r="O32" t="n">
         <v>370</v>
       </c>
+      <c r="S32" t="n">
+        <v>15</v>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>alpa</t>
+        </is>
+      </c>
+      <c r="U32" t="n">
+        <v>525</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2944,6 +3237,17 @@
       <c r="O33" t="n">
         <v>325</v>
       </c>
+      <c r="S33" t="n">
+        <v>16</v>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>PlusMicron</t>
+        </is>
+      </c>
+      <c r="U33" t="n">
+        <v>515</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2979,6 +3283,17 @@
       <c r="O34" t="n">
         <v>315</v>
       </c>
+      <c r="S34" t="n">
+        <v>17</v>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>Akane</t>
+        </is>
+      </c>
+      <c r="U34" t="n">
+        <v>485</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -3014,6 +3329,17 @@
       <c r="O35" t="n">
         <v>300</v>
       </c>
+      <c r="S35" t="n">
+        <v>18</v>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>Hi Im Yolo</t>
+        </is>
+      </c>
+      <c r="U35" t="n">
+        <v>485</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -3049,6 +3375,17 @@
       <c r="O36" t="n">
         <v>285</v>
       </c>
+      <c r="S36" t="n">
+        <v>19</v>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>timesprout</t>
+        </is>
+      </c>
+      <c r="U36" t="n">
+        <v>475</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -3084,6 +3421,17 @@
       <c r="O37" t="n">
         <v>215</v>
       </c>
+      <c r="S37" t="n">
+        <v>20</v>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>Hellmet</t>
+        </is>
+      </c>
+      <c r="U37" t="n">
+        <v>470</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -3119,6 +3467,17 @@
       <c r="O38" t="n">
         <v>90</v>
       </c>
+      <c r="S38" t="n">
+        <v>21</v>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>Samueras</t>
+        </is>
+      </c>
+      <c r="U38" t="n">
+        <v>305</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -3154,6 +3513,17 @@
       <c r="O39" t="n">
         <v>90</v>
       </c>
+      <c r="S39" t="n">
+        <v>22</v>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>Six</t>
+        </is>
+      </c>
+      <c r="U39" t="n">
+        <v>270</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -3189,6 +3559,17 @@
       <c r="O40" t="n">
         <v>60</v>
       </c>
+      <c r="S40" t="n">
+        <v>23</v>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>M4DSCOTSM4N</t>
+        </is>
+      </c>
+      <c r="U40" t="n">
+        <v>240</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -3224,6 +3605,17 @@
       <c r="O41" t="n">
         <v>30</v>
       </c>
+      <c r="S41" t="n">
+        <v>24</v>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>liz1rd</t>
+        </is>
+      </c>
+      <c r="U41" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -3253,6 +3645,11 @@
           <t>Nuisance</t>
         </is>
       </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>Nuisance</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -3282,6 +3679,17 @@
       <c r="O43" t="n">
         <v>860</v>
       </c>
+      <c r="S43" t="n">
+        <v>1</v>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>justMaki</t>
+        </is>
+      </c>
+      <c r="U43" t="n">
+        <v>900</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -3317,6 +3725,17 @@
       <c r="O44" t="n">
         <v>485</v>
       </c>
+      <c r="S44" t="n">
+        <v>2</v>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>IronDragon111000</t>
+        </is>
+      </c>
+      <c r="U44" t="n">
+        <v>355</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -3351,6 +3770,17 @@
       </c>
       <c r="O45" t="n">
         <v>370</v>
+      </c>
+      <c r="S45" t="n">
+        <v>3</v>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>brrryy</t>
+        </is>
+      </c>
+      <c r="U45" t="n">
+        <v>170</v>
       </c>
     </row>
     <row r="46">

</xml_diff>